<commit_message>
co2_pipelines_oeuvray.py, MEA, CPUs and node_metrics.xlsx updated
</commit_message>
<xml_diff>
--- a/southern_europe/northern_italy_data/geographical_feature/node_metrics.xlsx
+++ b/southern_europe/northern_italy_data/geographical_feature/node_metrics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mockp\PycharmProjects\AdOpT-NET0_XiaoY\southern_europe\northern_italy_data\geographical_feature\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7676ABD7-8CE3-4FB6-9BC2-4EDBEC7045A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD20363E-53CE-4E68-B842-DF39DE55C5A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{91043432-DB94-1942-B1A7-90AE2913C3A6}"/>
+    <workbookView xWindow="-5295" yWindow="-21720" windowWidth="38640" windowHeight="21120" xr2:uid="{91043432-DB94-1942-B1A7-90AE2913C3A6}"/>
   </bookViews>
   <sheets>
     <sheet name="nodes" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="186">
   <si>
     <t>Source</t>
   </si>
@@ -580,9 +580,6 @@
   </si>
   <si>
     <t>Ravenna</t>
-  </si>
-  <si>
-    <t>Other</t>
   </si>
   <si>
     <t>Reference Year</t>
@@ -1104,13 +1101,13 @@
         <v>143</v>
       </c>
       <c r="E1" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F1" s="15" t="s">
         <v>144</v>
       </c>
       <c r="G1" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>174</v>
@@ -1218,7 +1215,7 @@
       </c>
       <c r="G5" s="15"/>
       <c r="H5" s="1" t="s">
-        <v>2</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
@@ -1266,7 +1263,7 @@
       </c>
       <c r="G7" s="15"/>
       <c r="H7" s="1" t="s">
-        <v>2</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
@@ -1293,7 +1290,7 @@
         <v>587138469.99999881</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>2</v>
+        <v>52</v>
       </c>
       <c r="J8" s="12"/>
       <c r="K8" s="10"/>
@@ -1421,7 +1418,7 @@
       </c>
       <c r="G13" s="15"/>
       <c r="H13" s="1" t="s">
-        <v>2</v>
+        <v>52</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
@@ -1445,7 +1442,7 @@
       </c>
       <c r="G14" s="15"/>
       <c r="H14" s="1" t="s">
-        <v>179</v>
+        <v>52</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
@@ -1453,7 +1450,7 @@
         <v>13</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C15" s="14">
         <v>12.274480000000001</v>
@@ -5316,7 +5313,7 @@
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B42" s="15">
         <v>2024</v>
@@ -5324,7 +5321,7 @@
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B43">
         <v>288</v>
@@ -5332,7 +5329,7 @@
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B44" s="24">
         <f>28.9/AVERAGE(railway!C2,railway!D3,railway!F4,railway!M10)+0.07</f>
@@ -5341,7 +5338,7 @@
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B45" s="24">
         <f>5.58/AVERAGE(truck!C2,truck!D3,truck!E4,truck!F4,truck!F5,truck!G6,truck!F11,truck!F12,truck!I7,truck!I10,truck!I12,truck!J7,truck!J8,truck!J9,truck!J12,truck!K2,truck!K3,truck!K4,truck!L2,truck!L5,truck!L6,truck!L8,truck!L11,truck!M9,truck!M10,truck!N9,truck!N10,truck!N13)+0.15</f>

</xml_diff>

<commit_message>
main.py, ccs.py and MEA adapted; design updates 2ndFinal version
</commit_message>
<xml_diff>
--- a/southern_europe/northern_italy_data/geographical_feature/node_metrics.xlsx
+++ b/southern_europe/northern_italy_data/geographical_feature/node_metrics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mockp\PycharmProjects\AdOpT-NET0_XiaoY\southern_europe\northern_italy_data\geographical_feature\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7676ABD7-8CE3-4FB6-9BC2-4EDBEC7045A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEF4CB6A-FD51-4FFE-A6FC-62493604B417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{91043432-DB94-1942-B1A7-90AE2913C3A6}"/>
+    <workbookView xWindow="-5295" yWindow="-21720" windowWidth="38640" windowHeight="21120" xr2:uid="{91043432-DB94-1942-B1A7-90AE2913C3A6}"/>
   </bookViews>
   <sheets>
     <sheet name="nodes" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="186">
   <si>
     <t>Source</t>
   </si>
@@ -580,9 +580,6 @@
   </si>
   <si>
     <t>Ravenna</t>
-  </si>
-  <si>
-    <t>Other</t>
   </si>
   <si>
     <t>Reference Year</t>
@@ -1104,13 +1101,13 @@
         <v>143</v>
       </c>
       <c r="E1" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F1" s="15" t="s">
         <v>144</v>
       </c>
       <c r="G1" s="15" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>174</v>
@@ -1218,7 +1215,7 @@
       </c>
       <c r="G5" s="15"/>
       <c r="H5" s="1" t="s">
-        <v>2</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
@@ -1266,7 +1263,7 @@
       </c>
       <c r="G7" s="15"/>
       <c r="H7" s="1" t="s">
-        <v>2</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
@@ -1293,7 +1290,7 @@
         <v>587138469.99999881</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>2</v>
+        <v>52</v>
       </c>
       <c r="J8" s="12"/>
       <c r="K8" s="10"/>
@@ -1421,7 +1418,7 @@
       </c>
       <c r="G13" s="15"/>
       <c r="H13" s="1" t="s">
-        <v>2</v>
+        <v>52</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
@@ -1445,7 +1442,7 @@
       </c>
       <c r="G14" s="15"/>
       <c r="H14" s="1" t="s">
-        <v>179</v>
+        <v>52</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
@@ -1453,7 +1450,7 @@
         <v>13</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C15" s="14">
         <v>12.274480000000001</v>
@@ -5316,7 +5313,7 @@
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B42" s="15">
         <v>2024</v>
@@ -5324,7 +5321,7 @@
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B43">
         <v>288</v>
@@ -5332,7 +5329,7 @@
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B44" s="24">
         <f>28.9/AVERAGE(railway!C2,railway!D3,railway!F4,railway!M10)+0.07</f>
@@ -5341,7 +5338,7 @@
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B45" s="24">
         <f>5.58/AVERAGE(truck!C2,truck!D3,truck!E4,truck!F4,truck!F5,truck!G6,truck!F11,truck!F12,truck!I7,truck!I10,truck!I12,truck!J7,truck!J8,truck!J9,truck!J12,truck!K2,truck!K3,truck!K4,truck!L2,truck!L5,truck!L6,truck!L8,truck!L11,truck!M9,truck!M10,truck!N9,truck!N10,truck!N13)+0.15</f>

</xml_diff>